<commit_message>
learning pysystemtrade. added comparison for long-short vs long-only, vs buy and hold IVV and HYD
</commit_message>
<xml_diff>
--- a/perplexity_examples/cash_weights_time_series.xlsx
+++ b/perplexity_examples/cash_weights_time_series.xlsx
@@ -614,28 +614,28 @@
         <v>0.06747301079568173</v>
       </c>
       <c r="C2">
-        <v>0.6976300517174882</v>
+        <v>0.6976300627326517</v>
       </c>
       <c r="D2">
-        <v>0.1107453374381761</v>
+        <v>0.1107453391867791</v>
       </c>
       <c r="E2">
         <v>0.12</v>
       </c>
       <c r="F2">
-        <v>1.083567062739687</v>
+        <v>1.083567045630808</v>
       </c>
       <c r="G2">
-        <v>0.07311153212208002</v>
+        <v>0.07311153096769245</v>
       </c>
       <c r="H2">
-        <v>1.083567062739687</v>
+        <v>1.083567045630808</v>
       </c>
       <c r="I2">
-        <v>0.08356706273968673</v>
+        <v>0.08356704563080775</v>
       </c>
       <c r="J2">
-        <v>0.005638521326398291</v>
+        <v>0.005638520172010719</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -646,28 +646,28 @@
         <v>0.08506597361055578</v>
       </c>
       <c r="C3">
-        <v>0.4560689073104038</v>
+        <v>0.4560689137162595</v>
       </c>
       <c r="D3">
-        <v>0.07239869456713778</v>
+        <v>0.07239869558403583</v>
       </c>
       <c r="E3">
         <v>0.12</v>
       </c>
       <c r="F3">
-        <v>1.657488449446003</v>
+        <v>1.657488426165242</v>
       </c>
       <c r="G3">
-        <v>0.1409958687003747</v>
+        <v>0.1409958667199741</v>
       </c>
       <c r="H3">
-        <v>1.657488449446003</v>
+        <v>1.657488426165242</v>
       </c>
       <c r="I3">
-        <v>0.6574884494460034</v>
+        <v>0.6574884261652418</v>
       </c>
       <c r="J3">
-        <v>0.05592989508981895</v>
+        <v>0.0559298931094183</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -678,28 +678,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C4">
-        <v>0.2269870542221717</v>
+        <v>0.2269865387852764</v>
       </c>
       <c r="D4">
-        <v>0.03603307777818001</v>
+        <v>0.03603299595510951</v>
       </c>
       <c r="E4">
         <v>0.12</v>
       </c>
       <c r="F4">
-        <v>3.330273387655676</v>
+        <v>3.330280949979789</v>
       </c>
       <c r="G4">
-        <v>0.01830917996012217</v>
+        <v>0.01830922153627433</v>
       </c>
       <c r="H4">
-        <v>3.330273387655676</v>
+        <v>3.330280949979789</v>
       </c>
       <c r="I4">
-        <v>2.330273387655676</v>
+        <v>2.330280949979789</v>
       </c>
       <c r="J4">
-        <v>0.01281137908047403</v>
+        <v>0.01281142065662619</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -710,28 +710,28 @@
         <v>0.0505797680927629</v>
       </c>
       <c r="C5">
-        <v>0.3313947854214608</v>
+        <v>0.3313942477011748</v>
       </c>
       <c r="D5">
-        <v>0.05260729128052791</v>
+        <v>0.05260720592007881</v>
       </c>
       <c r="E5">
         <v>0.12</v>
       </c>
       <c r="F5">
-        <v>2.281052627478976</v>
+        <v>2.281056328714829</v>
       </c>
       <c r="G5">
-        <v>0.1153751129052741</v>
+        <v>0.1153753001129252</v>
       </c>
       <c r="H5">
-        <v>2.281052627478976</v>
+        <v>2.281056328714829</v>
       </c>
       <c r="I5">
-        <v>1.281052627478976</v>
+        <v>1.281056328714829</v>
       </c>
       <c r="J5">
-        <v>0.06479534481251117</v>
+        <v>0.06479553202016231</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -742,28 +742,28 @@
         <v>0.01859256297481008</v>
       </c>
       <c r="C6">
-        <v>0.359105752617937</v>
+        <v>0.3591059303506379</v>
       </c>
       <c r="D6">
-        <v>0.0570062709479846</v>
+        <v>0.05700629916217619</v>
       </c>
       <c r="E6">
         <v>0.12</v>
       </c>
       <c r="F6">
-        <v>2.105031569412672</v>
+        <v>2.105030527567035</v>
       </c>
       <c r="G6">
-        <v>0.03913793201826839</v>
+        <v>0.03913791264768778</v>
       </c>
       <c r="H6">
-        <v>2.105031569412672</v>
+        <v>2.105030527567035</v>
       </c>
       <c r="I6">
-        <v>1.105031569412672</v>
+        <v>1.105030527567035</v>
       </c>
       <c r="J6">
-        <v>0.02054536904345831</v>
+        <v>0.02054534967287771</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -774,28 +774,28 @@
         <v>0.01859256297481008</v>
       </c>
       <c r="C7">
-        <v>0.3525081487940714</v>
+        <v>0.3525083045506299</v>
       </c>
       <c r="D7">
-        <v>0.05595893380997197</v>
+        <v>0.0559589585355591</v>
       </c>
       <c r="E7">
         <v>0.12</v>
       </c>
       <c r="F7">
-        <v>2.14442970638972</v>
+        <v>2.144428758868806</v>
       </c>
       <c r="G7">
-        <v>0.03987044436110435</v>
+        <v>0.0398704267442621</v>
       </c>
       <c r="H7">
-        <v>2.14442970638972</v>
+        <v>2.144428758868806</v>
       </c>
       <c r="I7">
-        <v>1.14442970638972</v>
+        <v>1.144428758868806</v>
       </c>
       <c r="J7">
-        <v>0.02127788138629428</v>
+        <v>0.02127786376945202</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -806,28 +806,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C8">
-        <v>1.131066338203995</v>
+        <v>1.131066377339455</v>
       </c>
       <c r="D8">
-        <v>0.1795512148322547</v>
+        <v>0.1795512210448164</v>
       </c>
       <c r="E8">
         <v>0.12</v>
       </c>
       <c r="F8">
-        <v>0.6683329885131086</v>
+        <v>0.6683329653884545</v>
       </c>
       <c r="G8">
-        <v>0.007549143112952946</v>
+        <v>0.007549142851748836</v>
       </c>
       <c r="H8">
-        <v>0.6683329885131086</v>
+        <v>0.6683329653884545</v>
       </c>
       <c r="I8">
-        <v>-0.3316670114868914</v>
+        <v>-0.3316670346115455</v>
       </c>
       <c r="J8">
-        <v>-0.003746338694324143</v>
+        <v>-0.003746338955528252</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -838,28 +838,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C9">
-        <v>1.078262861777704</v>
+        <v>1.078262870730279</v>
       </c>
       <c r="D9">
-        <v>0.1711689228132371</v>
+        <v>0.1711689242344143</v>
       </c>
       <c r="E9">
         <v>0.12</v>
       </c>
       <c r="F9">
-        <v>0.7010618401269743</v>
+        <v>0.7010618343062149</v>
       </c>
       <c r="G9">
-        <v>0.007918831260930436</v>
+        <v>0.007918831195182155</v>
       </c>
       <c r="H9">
-        <v>0.7010618401269743</v>
+        <v>0.7010618343062149</v>
       </c>
       <c r="I9">
-        <v>-0.2989381598730257</v>
+        <v>-0.2989381656937851</v>
       </c>
       <c r="J9">
-        <v>-0.003376650546346652</v>
+        <v>-0.003376650612094934</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -870,28 +870,28 @@
         <v>0.02249100359856058</v>
       </c>
       <c r="C10">
-        <v>0.5926632641986557</v>
+        <v>0.5926633558141835</v>
       </c>
       <c r="D10">
-        <v>0.09408237649640477</v>
+        <v>0.09408239103991896</v>
       </c>
       <c r="E10">
         <v>0.12</v>
       </c>
       <c r="F10">
-        <v>1.275477985025024</v>
+        <v>1.275477787858136</v>
       </c>
       <c r="G10">
-        <v>0.02868677995108259</v>
+        <v>0.02868677551660143</v>
       </c>
       <c r="H10">
-        <v>1.275477985025024</v>
+        <v>1.275477787858136</v>
       </c>
       <c r="I10">
-        <v>0.2754779850250235</v>
+        <v>0.2754777878581365</v>
       </c>
       <c r="J10">
-        <v>0.006195776352522019</v>
+        <v>0.006195771918040854</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -902,28 +902,28 @@
         <v>0.04498200719712115</v>
       </c>
       <c r="C11">
-        <v>0.820544382965599</v>
+        <v>0.8205444223118962</v>
       </c>
       <c r="D11">
-        <v>0.1302573826210751</v>
+        <v>0.1302573888671062</v>
       </c>
       <c r="E11">
         <v>0.12</v>
       </c>
       <c r="F11">
-        <v>0.9212529653623215</v>
+        <v>0.9212529211869033</v>
       </c>
       <c r="G11">
-        <v>0.04143980751829714</v>
+        <v>0.04143980553119817</v>
       </c>
       <c r="H11">
-        <v>0.9212529653623215</v>
+        <v>0.9212529211869033</v>
       </c>
       <c r="I11">
-        <v>-0.07874703463767851</v>
+        <v>-0.07874707881309673</v>
       </c>
       <c r="J11">
-        <v>-0.003542199678824007</v>
+        <v>-0.003542201665922985</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -934,28 +934,28 @@
         <v>0.007297081167532987</v>
       </c>
       <c r="C12">
-        <v>0.2918383850730365</v>
+        <v>0.2918384780843121</v>
       </c>
       <c r="D12">
-        <v>0.04632790739555755</v>
+        <v>0.04632792216063981</v>
       </c>
       <c r="E12">
         <v>0.12</v>
       </c>
       <c r="F12">
-        <v>2.590231390669438</v>
+        <v>2.590230565141813</v>
       </c>
       <c r="G12">
-        <v>0.01890112870040674</v>
+        <v>0.01890112267646465</v>
       </c>
       <c r="H12">
-        <v>2.590231390669438</v>
+        <v>2.590230565141813</v>
       </c>
       <c r="I12">
-        <v>1.590231390669438</v>
+        <v>1.590230565141813</v>
       </c>
       <c r="J12">
-        <v>0.01160404753287375</v>
+        <v>0.01160404150893166</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -966,28 +966,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C13">
-        <v>0.2235623731374612</v>
+        <v>0.2235623682645147</v>
       </c>
       <c r="D13">
-        <v>0.03548942650998895</v>
+        <v>0.03548942573643268</v>
       </c>
       <c r="E13">
         <v>0.12</v>
       </c>
       <c r="F13">
-        <v>3.381288789387015</v>
+        <v>3.381288863088324</v>
       </c>
       <c r="G13">
-        <v>0.01858965248063633</v>
+        <v>0.01858965288583145</v>
       </c>
       <c r="H13">
-        <v>3.381288789387015</v>
+        <v>3.381288863088324</v>
       </c>
       <c r="I13">
-        <v>2.381288789387015</v>
+        <v>2.381288863088324</v>
       </c>
       <c r="J13">
-        <v>0.01309185160098819</v>
+        <v>0.01309185200618331</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1030,28 +1030,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C15">
-        <v>0.5262364732925436</v>
+        <v>0.526236344574488</v>
       </c>
       <c r="D15">
-        <v>0.08353745034862524</v>
+        <v>0.08353742991526734</v>
       </c>
       <c r="E15">
         <v>0.12</v>
       </c>
       <c r="F15">
-        <v>1.436481476262518</v>
+        <v>1.436481827627651</v>
       </c>
       <c r="G15">
-        <v>0.007897489123794331</v>
+        <v>0.007897491055529865</v>
       </c>
       <c r="H15">
-        <v>1.436481476262518</v>
+        <v>1.436481827627651</v>
       </c>
       <c r="I15">
-        <v>0.4364814762625182</v>
+        <v>0.4364818276276505</v>
       </c>
       <c r="J15">
-        <v>0.002399688244146191</v>
+        <v>0.002399690175881724</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1062,28 +1062,28 @@
         <v>0.04498200719712115</v>
       </c>
       <c r="C16">
-        <v>0.6165504959464999</v>
+        <v>0.6165504471811983</v>
       </c>
       <c r="D16">
-        <v>0.09787435697927854</v>
+        <v>0.0978743492380269</v>
       </c>
       <c r="E16">
         <v>0.12</v>
       </c>
       <c r="F16">
-        <v>1.226061694846238</v>
+        <v>1.226061791820085</v>
       </c>
       <c r="G16">
-        <v>0.05515071598168804</v>
+        <v>0.0551507203437663</v>
       </c>
       <c r="H16">
-        <v>1.226061694846238</v>
+        <v>1.226061791820085</v>
       </c>
       <c r="I16">
-        <v>0.2260616948462382</v>
+        <v>0.2260617918200847</v>
       </c>
       <c r="J16">
-        <v>0.01016870878456689</v>
+        <v>0.01016871314664515</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1094,28 +1094,28 @@
         <v>0.06377449020391843</v>
       </c>
       <c r="C17">
-        <v>0.3045119029789629</v>
+        <v>0.3045122453909766</v>
       </c>
       <c r="D17">
-        <v>0.04833976599248188</v>
+        <v>0.04833982034870393</v>
       </c>
       <c r="E17">
         <v>0.12</v>
       </c>
       <c r="F17">
-        <v>2.482428235557929</v>
+        <v>2.482425444165255</v>
       </c>
       <c r="G17">
-        <v>0.1583155951905197</v>
+        <v>0.1583154171708749</v>
       </c>
       <c r="H17">
-        <v>2.482428235557929</v>
+        <v>2.482425444165255</v>
       </c>
       <c r="I17">
-        <v>1.482428235557929</v>
+        <v>1.482425444165255</v>
       </c>
       <c r="J17">
-        <v>0.09454110498660123</v>
+        <v>0.09454092696695651</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1126,28 +1126,28 @@
         <v>0.03378648540583766</v>
       </c>
       <c r="C18">
-        <v>0.9486096880270347</v>
+        <v>0.9486097644190314</v>
       </c>
       <c r="D18">
-        <v>0.150587119547166</v>
+        <v>0.1505871316740195</v>
       </c>
       <c r="E18">
         <v>0.12</v>
       </c>
       <c r="F18">
-        <v>0.7968809042954987</v>
+        <v>0.7968808401222995</v>
       </c>
       <c r="G18">
-        <v>0.02692380504317058</v>
+        <v>0.02692380287498373</v>
       </c>
       <c r="H18">
-        <v>0.7968809042954987</v>
+        <v>0.7968808401222995</v>
       </c>
       <c r="I18">
-        <v>-0.2031190957045013</v>
+        <v>-0.2031191598777005</v>
       </c>
       <c r="J18">
-        <v>-0.006862680362667076</v>
+        <v>-0.006862682530853932</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1158,28 +1158,28 @@
         <v>0.0899640143942423</v>
       </c>
       <c r="C19">
-        <v>0.5603449438008412</v>
+        <v>0.560344939860325</v>
       </c>
       <c r="D19">
-        <v>0.08895200218256941</v>
+        <v>0.08895200155703184</v>
       </c>
       <c r="E19">
         <v>0.12</v>
       </c>
       <c r="F19">
-        <v>1.349042146951411</v>
+        <v>1.349042156438286</v>
       </c>
       <c r="G19">
-        <v>0.1213652471267763</v>
+        <v>0.1213652479802536</v>
       </c>
       <c r="H19">
-        <v>1.349042146951411</v>
+        <v>1.349042156438286</v>
       </c>
       <c r="I19">
-        <v>0.3490421469514107</v>
+        <v>0.349042156438286</v>
       </c>
       <c r="J19">
-        <v>0.03140123273253395</v>
+        <v>0.03140123358601134</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1190,28 +1190,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C20">
-        <v>1.23744385730069</v>
+        <v>1.237443723167047</v>
       </c>
       <c r="D20">
-        <v>0.1964381224693274</v>
+        <v>0.1964381011762718</v>
       </c>
       <c r="E20">
         <v>0.12</v>
       </c>
       <c r="F20">
-        <v>0.6108793878272647</v>
+        <v>0.610879454043995</v>
       </c>
       <c r="G20">
-        <v>0.006900177011643433</v>
+        <v>0.006900177759593306</v>
       </c>
       <c r="H20">
-        <v>0.6108793878272647</v>
+        <v>0.610879454043995</v>
       </c>
       <c r="I20">
-        <v>-0.3891206121727353</v>
+        <v>-0.389120545956005</v>
       </c>
       <c r="J20">
-        <v>-0.004395304795633655</v>
+        <v>-0.004395304047683782</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1222,28 +1222,28 @@
         <v>0.06377449020391843</v>
       </c>
       <c r="C21">
-        <v>0.4690631565455226</v>
+        <v>0.4690632766710807</v>
       </c>
       <c r="D21">
-        <v>0.0744614676841447</v>
+        <v>0.07446148675348588</v>
       </c>
       <c r="E21">
         <v>0.12</v>
       </c>
       <c r="F21">
-        <v>1.611571779769685</v>
+        <v>1.611571367051468</v>
       </c>
       <c r="G21">
-        <v>0.1027771686818332</v>
+        <v>0.1027771423609393</v>
       </c>
       <c r="H21">
-        <v>1.611571779769685</v>
+        <v>1.611571367051468</v>
       </c>
       <c r="I21">
-        <v>0.6115717797696854</v>
+        <v>0.6115713670514678</v>
       </c>
       <c r="J21">
-        <v>0.03900267847791476</v>
+        <v>0.03900265215702083</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1254,28 +1254,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C22">
-        <v>0.09215783482745128</v>
+        <v>0.092157954800765</v>
       </c>
       <c r="D22">
-        <v>0.01462960273917619</v>
+        <v>0.01462962178434932</v>
       </c>
       <c r="E22">
         <v>0.12</v>
       </c>
       <c r="F22">
-        <v>8.202546722520047</v>
+        <v>8.202536044258869</v>
       </c>
       <c r="G22">
-        <v>0.07461332984299525</v>
+        <v>0.07461323270967185</v>
       </c>
       <c r="H22">
-        <v>8.202546722520047</v>
+        <v>8.202536044258869</v>
       </c>
       <c r="I22">
-        <v>7.202546722520047</v>
+        <v>7.202536044258869</v>
       </c>
       <c r="J22">
-        <v>0.06551696838757741</v>
+        <v>0.06551687125425401</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1286,28 +1286,28 @@
         <v>0.01009596161535386</v>
       </c>
       <c r="C23">
-        <v>0.2279696537070912</v>
+        <v>0.2279697461151154</v>
       </c>
       <c r="D23">
-        <v>0.03618906061070863</v>
+        <v>0.0361890752800277</v>
       </c>
       <c r="E23">
         <v>0.12</v>
       </c>
       <c r="F23">
-        <v>3.315919174881568</v>
+        <v>3.315917830766637</v>
       </c>
       <c r="G23">
-        <v>0.03347739270922014</v>
+        <v>0.0334773791390874</v>
       </c>
       <c r="H23">
-        <v>3.315919174881568</v>
+        <v>3.315917830766637</v>
       </c>
       <c r="I23">
-        <v>2.315919174881568</v>
+        <v>2.315917830766637</v>
       </c>
       <c r="J23">
-        <v>0.02338143109386628</v>
+        <v>0.02338141752373354</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1318,28 +1318,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C24">
-        <v>0.2133665889835189</v>
+        <v>0.213366366214786</v>
       </c>
       <c r="D24">
-        <v>0.03387089595243149</v>
+        <v>0.03387086058899146</v>
       </c>
       <c r="E24">
         <v>0.12</v>
       </c>
       <c r="F24">
-        <v>3.542864651957503</v>
+        <v>3.542868350944758</v>
       </c>
       <c r="G24">
-        <v>0.03222717746182855</v>
+        <v>0.03222721110915364</v>
       </c>
       <c r="H24">
-        <v>3.542864651957503</v>
+        <v>3.542868350944758</v>
       </c>
       <c r="I24">
-        <v>2.542864651957503</v>
+        <v>2.542868350944758</v>
       </c>
       <c r="J24">
-        <v>0.02313081600641072</v>
+        <v>0.02313084965373581</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1350,28 +1350,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C25">
-        <v>0.2067751902284032</v>
+        <v>0.2067753155382149</v>
       </c>
       <c r="D25">
-        <v>0.03282454383854568</v>
+        <v>0.03282456373086159</v>
       </c>
       <c r="E25">
         <v>0.12</v>
       </c>
       <c r="F25">
-        <v>3.655800994226908</v>
+        <v>3.655798778741307</v>
       </c>
       <c r="G25">
-        <v>0.02009886592187924</v>
+        <v>0.02009885374158056</v>
       </c>
       <c r="H25">
-        <v>3.655800994226908</v>
+        <v>3.655798778741307</v>
       </c>
       <c r="I25">
-        <v>2.655800994226908</v>
+        <v>2.655798778741307</v>
       </c>
       <c r="J25">
-        <v>0.0146010650422311</v>
+        <v>0.01460105286193242</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1382,28 +1382,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C26">
-        <v>0.09228877500229649</v>
+        <v>0.09228875420481907</v>
       </c>
       <c r="D26">
-        <v>0.01465038884753226</v>
+        <v>0.01465038554603507</v>
       </c>
       <c r="E26">
         <v>0.12</v>
       </c>
       <c r="F26">
-        <v>8.19090887271658</v>
+        <v>8.190910718556236</v>
       </c>
       <c r="G26">
-        <v>0.07450746775461904</v>
+        <v>0.07450748454504375</v>
       </c>
       <c r="H26">
-        <v>8.19090887271658</v>
+        <v>8.190910718556236</v>
       </c>
       <c r="I26">
-        <v>7.19090887271658</v>
+        <v>7.190910718556236</v>
       </c>
       <c r="J26">
-        <v>0.0654111062992012</v>
+        <v>0.06541112308962591</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -1414,28 +1414,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C27">
-        <v>0.6474560812431809</v>
+        <v>0.6474564107116441</v>
       </c>
       <c r="D27">
-        <v>0.1027804665483533</v>
+        <v>0.1027805188498504</v>
       </c>
       <c r="E27">
         <v>0.12</v>
       </c>
       <c r="F27">
-        <v>1.167537023618644</v>
+        <v>1.167536429498913</v>
       </c>
       <c r="G27">
-        <v>0.0106203387794179</v>
+        <v>0.01062033337509007</v>
       </c>
       <c r="H27">
-        <v>1.167537023618644</v>
+        <v>1.167536429498913</v>
       </c>
       <c r="I27">
-        <v>0.1675370236186442</v>
+        <v>0.1675364294989128</v>
       </c>
       <c r="J27">
-        <v>0.001523977324000062</v>
+        <v>0.001523971919672238</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -1446,28 +1446,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C28">
-        <v>0.2536538907219163</v>
+        <v>0.2536535886882946</v>
       </c>
       <c r="D28">
-        <v>0.04026630683604867</v>
+        <v>0.04026625888969763</v>
       </c>
       <c r="E28">
         <v>0.12</v>
       </c>
       <c r="F28">
-        <v>2.980159081601425</v>
+        <v>2.980162630174286</v>
       </c>
       <c r="G28">
-        <v>0.02710860420089262</v>
+        <v>0.027108636479994</v>
       </c>
       <c r="H28">
-        <v>2.980159081601425</v>
+        <v>2.980162630174286</v>
       </c>
       <c r="I28">
-        <v>1.980159081601425</v>
+        <v>1.980162630174286</v>
       </c>
       <c r="J28">
-        <v>0.01801224274547478</v>
+        <v>0.01801227502457617</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1478,28 +1478,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C29">
-        <v>0.5223999155527357</v>
+        <v>0.5223999582569488</v>
       </c>
       <c r="D29">
-        <v>0.08292841568842091</v>
+        <v>0.08292842246750459</v>
       </c>
       <c r="E29">
         <v>0.12</v>
       </c>
       <c r="F29">
-        <v>1.447031141302212</v>
+        <v>1.44703102301291</v>
       </c>
       <c r="G29">
-        <v>0.01316271829853072</v>
+        <v>0.01316271722252848</v>
       </c>
       <c r="H29">
-        <v>1.447031141302212</v>
+        <v>1.44703102301291</v>
       </c>
       <c r="I29">
-        <v>0.4470311413022123</v>
+        <v>0.4470310230129104</v>
       </c>
       <c r="J29">
-        <v>0.004066356843112887</v>
+        <v>0.004066355767110641</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1510,28 +1510,28 @@
         <v>0.1124550179928029</v>
       </c>
       <c r="C30">
-        <v>0.6675113988665514</v>
+        <v>0.667511455493796</v>
       </c>
       <c r="D30">
-        <v>0.1059641495221042</v>
+        <v>0.1059641585114006</v>
       </c>
       <c r="E30">
         <v>0.12</v>
       </c>
       <c r="F30">
-        <v>1.132458482809489</v>
+        <v>1.132458386739222</v>
       </c>
       <c r="G30">
-        <v>0.1273506390604433</v>
+        <v>0.1273506282568598</v>
       </c>
       <c r="H30">
-        <v>1.132458482809489</v>
+        <v>1.132458386739222</v>
       </c>
       <c r="I30">
-        <v>0.1324584828094888</v>
+        <v>0.1324583867392224</v>
       </c>
       <c r="J30">
-        <v>0.01489562106764045</v>
+        <v>0.01489561026405689</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -1542,28 +1542,28 @@
         <v>0.007297081167532987</v>
       </c>
       <c r="C31">
-        <v>0.2635346237431639</v>
+        <v>0.2635345622274512</v>
       </c>
       <c r="D31">
-        <v>0.04183482457676337</v>
+        <v>0.04183481481144672</v>
       </c>
       <c r="E31">
         <v>0.12</v>
       </c>
       <c r="F31">
-        <v>2.868423644990076</v>
+        <v>2.86842431455358</v>
       </c>
       <c r="G31">
-        <v>0.02093112016036341</v>
+        <v>0.02093112504622264</v>
       </c>
       <c r="H31">
-        <v>2.868423644990076</v>
+        <v>2.86842431455358</v>
       </c>
       <c r="I31">
-        <v>1.868423644990076</v>
+        <v>1.86842431455358</v>
       </c>
       <c r="J31">
-        <v>0.01363403899283042</v>
+        <v>0.01363404387868965</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1574,28 +1574,28 @@
         <v>0.02479008396641344</v>
       </c>
       <c r="C32">
-        <v>0.3171648145139504</v>
+        <v>0.3171650998878429</v>
       </c>
       <c r="D32">
-        <v>0.05034835342943052</v>
+        <v>0.05034839873113153</v>
       </c>
       <c r="E32">
         <v>0.12</v>
       </c>
       <c r="F32">
-        <v>2.383394725473891</v>
+        <v>2.383392580979965</v>
       </c>
       <c r="G32">
-        <v>0.05908455536960466</v>
+        <v>0.05908450220742018</v>
       </c>
       <c r="H32">
-        <v>2.383394725473891</v>
+        <v>2.383392580979965</v>
       </c>
       <c r="I32">
-        <v>1.383394725473891</v>
+        <v>1.383392580979965</v>
       </c>
       <c r="J32">
-        <v>0.03429447140319122</v>
+        <v>0.03429441824100674</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1606,28 +1606,28 @@
         <v>0.0235905637744902</v>
       </c>
       <c r="C33">
-        <v>0.5146400303751995</v>
+        <v>0.5146398445935794</v>
       </c>
       <c r="D33">
-        <v>0.08169657210549028</v>
+        <v>0.0816965426135724</v>
       </c>
       <c r="E33">
         <v>0.12</v>
       </c>
       <c r="F33">
-        <v>1.468849878365161</v>
+        <v>1.468850408610366</v>
       </c>
       <c r="G33">
-        <v>0.0346509967307255</v>
+        <v>0.03465100923950883</v>
       </c>
       <c r="H33">
-        <v>1.468849878365161</v>
+        <v>1.468850408610366</v>
       </c>
       <c r="I33">
-        <v>0.4688498783651609</v>
+        <v>0.468850408610366</v>
       </c>
       <c r="J33">
-        <v>0.0110604329562353</v>
+        <v>0.01106044546501863</v>
       </c>
     </row>
   </sheetData>
@@ -23913,7 +23913,7 @@
         <v>45796</v>
       </c>
       <c r="B2">
-        <v>1485035.449893672</v>
+        <v>1473655.975420408</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -23921,7 +23921,7 @@
         <v>45797</v>
       </c>
       <c r="B3">
-        <v>1486769.501859221</v>
+        <v>1475390.072551022</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -23929,7 +23929,7 @@
         <v>45798</v>
       </c>
       <c r="B4">
-        <v>1478792.339165517</v>
+        <v>1467412.805224441</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -23937,7 +23937,7 @@
         <v>45799</v>
       </c>
       <c r="B5">
-        <v>1479021.132175939</v>
+        <v>1467641.543772715</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -23945,7 +23945,7 @@
         <v>45800</v>
       </c>
       <c r="B6">
-        <v>1485333.716816519</v>
+        <v>1473954.784457617</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -23953,7 +23953,7 @@
         <v>45803</v>
       </c>
       <c r="B7">
-        <v>1485311.88415717</v>
+        <v>1473932.943876973</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -23961,7 +23961,7 @@
         <v>45804</v>
       </c>
       <c r="B8">
-        <v>1489376.680908193</v>
+        <v>1477996.603617421</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -23969,7 +23969,7 @@
         <v>45805</v>
       </c>
       <c r="B9">
-        <v>1483634.962698302</v>
+        <v>1472254.643139277</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -23977,7 +23977,7 @@
         <v>45806</v>
       </c>
       <c r="B10">
-        <v>1491260.696938402</v>
+        <v>1479881.485676732</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -23985,7 +23985,7 @@
         <v>45807</v>
       </c>
       <c r="B11">
-        <v>1490851.434027301</v>
+        <v>1479472.34020478</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -23993,7 +23993,7 @@
         <v>45810</v>
       </c>
       <c r="B12">
-        <v>1501941.877923924</v>
+        <v>1490562.84111433</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -24001,7 +24001,7 @@
         <v>45811</v>
       </c>
       <c r="B13">
-        <v>1497732.197750224</v>
+        <v>1486353.220892737</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -24009,7 +24009,7 @@
         <v>45812</v>
       </c>
       <c r="B14">
-        <v>1506246.094008826</v>
+        <v>1494868.056723908</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -24017,7 +24017,7 @@
         <v>45813</v>
       </c>
       <c r="B15">
-        <v>1503646.834943574</v>
+        <v>1492268.732707514</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -24025,7 +24025,7 @@
         <v>45814</v>
       </c>
       <c r="B16">
-        <v>1500454.740113403</v>
+        <v>1489075.64730576</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -24033,7 +24033,7 @@
         <v>45817</v>
       </c>
       <c r="B17">
-        <v>1505480.204078704</v>
+        <v>1494101.474552918</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -24041,7 +24041,7 @@
         <v>45818</v>
       </c>
       <c r="B18">
-        <v>1511050.270906562</v>
+        <v>1499671.793804988</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -24049,7 +24049,7 @@
         <v>45819</v>
       </c>
       <c r="B19">
-        <v>1514281.929240987</v>
+        <v>1502903.664313073</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -24057,7 +24057,7 @@
         <v>45820</v>
       </c>
       <c r="B20">
-        <v>1526164.161901768</v>
+        <v>1514786.387599644</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -24065,7 +24065,7 @@
         <v>45821</v>
       </c>
       <c r="B21">
-        <v>1510308.885778795</v>
+        <v>1498930.767398155</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -24073,7 +24073,7 @@
         <v>45824</v>
       </c>
       <c r="B22">
-        <v>1515937.361628292</v>
+        <v>1504559.80707812</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -24081,7 +24081,7 @@
         <v>45825</v>
       </c>
       <c r="B23">
-        <v>1503740.373793554</v>
+        <v>1492362.372592059</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -24089,7 +24089,7 @@
         <v>45826</v>
       </c>
       <c r="B24">
-        <v>1503725.577683249</v>
+        <v>1492347.675571135</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -24097,7 +24097,7 @@
         <v>45827</v>
       </c>
       <c r="B25">
-        <v>1503706.351331285</v>
+        <v>1492328.439442766</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -24105,7 +24105,7 @@
         <v>45828</v>
       </c>
       <c r="B26">
-        <v>1502188.984793091</v>
+        <v>1490811.329415057</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -24113,7 +24113,7 @@
         <v>45831</v>
       </c>
       <c r="B27">
-        <v>1509093.392574063</v>
+        <v>1497715.777348043</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -24121,7 +24121,7 @@
         <v>45832</v>
       </c>
       <c r="B28">
-        <v>1516923.369965698</v>
+        <v>1505546.237030588</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -24129,7 +24129,7 @@
         <v>45833</v>
       </c>
       <c r="B29">
-        <v>1514321.864902801</v>
+        <v>1502944.580239103</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -24137,7 +24137,7 @@
         <v>45834</v>
       </c>
       <c r="B30">
-        <v>1525371.774483825</v>
+        <v>1513994.861918902</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -24145,7 +24145,7 @@
         <v>45835</v>
       </c>
       <c r="B31">
-        <v>1522849.558751748</v>
+        <v>1511472.57254864</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -24153,7 +24153,7 @@
         <v>45838</v>
       </c>
       <c r="B32">
-        <v>1535955.277272001</v>
+        <v>1524578.831275726</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -24161,7 +24161,7 @@
         <v>45839</v>
       </c>
       <c r="B33">
-        <v>1538485.467791676</v>
+        <v>1527109.022923371</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -24169,7 +24169,7 @@
         <v>45840</v>
       </c>
       <c r="B34">
-        <v>1538448.728399994</v>
+        <v>1527071.842841107</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -24177,7 +24177,7 @@
         <v>45841</v>
       </c>
       <c r="B35">
-        <v>1541268.559143565</v>
+        <v>1529891.633783187</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -24185,7 +24185,7 @@
         <v>45842</v>
       </c>
       <c r="B36">
-        <v>1541256.876147552</v>
+        <v>1529879.953039497</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -24193,7 +24193,7 @@
         <v>45845</v>
       </c>
       <c r="B37">
-        <v>1521545.067820606</v>
+        <v>1510167.894210919</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -24201,7 +24201,7 @@
         <v>45846</v>
       </c>
       <c r="B38">
-        <v>1521566.77390328</v>
+        <v>1510189.544039101</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -24209,7 +24209,7 @@
         <v>45847</v>
       </c>
       <c r="B39">
-        <v>1529573.907437771</v>
+        <v>1518197.277841107</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -24217,7 +24217,7 @@
         <v>45848</v>
       </c>
       <c r="B40">
-        <v>1529866.897880598</v>
+        <v>1518490.212749423</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -24225,7 +24225,7 @@
         <v>45849</v>
       </c>
       <c r="B41">
-        <v>1522438.194563169</v>
+        <v>1511060.212329831</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -24233,7 +24233,7 @@
         <v>45852</v>
       </c>
       <c r="B42">
-        <v>1523256.697879857</v>
+        <v>1511878.99765606</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -24241,7 +24241,7 @@
         <v>45853</v>
       </c>
       <c r="B43">
-        <v>1516685.245154236</v>
+        <v>1505307.508255846</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -24249,7 +24249,7 @@
         <v>45854</v>
       </c>
       <c r="B44">
-        <v>1520802.485988825</v>
+        <v>1509424.794220224</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -24257,7 +24257,7 @@
         <v>45855</v>
       </c>
       <c r="B45">
-        <v>1523675.422974737</v>
+        <v>1512298.060307698</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -24265,7 +24265,7 @@
         <v>45856</v>
       </c>
       <c r="B46">
-        <v>1524761.300484674</v>
+        <v>1513384.644997465</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -24273,7 +24273,7 @@
         <v>45859</v>
       </c>
       <c r="B47">
-        <v>1528605.374134197</v>
+        <v>1517228.834964787</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -24281,7 +24281,7 @@
         <v>45860</v>
       </c>
       <c r="B48">
-        <v>1533169.0782315</v>
+        <v>1521793.378538795</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -24289,7 +24289,7 @@
         <v>45861</v>
       </c>
       <c r="B49">
-        <v>1537725.986969382</v>
+        <v>1526350.244136101</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -24297,7 +24297,7 @@
         <v>45862</v>
       </c>
       <c r="B50">
-        <v>1531300.829768996</v>
+        <v>1519924.314011556</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -24305,7 +24305,7 @@
         <v>45863</v>
       </c>
       <c r="B51">
-        <v>1529454.653454583</v>
+        <v>1518078.268600035</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -24313,7 +24313,7 @@
         <v>45866</v>
       </c>
       <c r="B52">
-        <v>1514670.902500041</v>
+        <v>1503294.367526044</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -24321,7 +24321,7 @@
         <v>45867</v>
       </c>
       <c r="B53">
-        <v>1517510.494526228</v>
+        <v>1506134.378628545</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -24329,7 +24329,7 @@
         <v>45868</v>
       </c>
       <c r="B54">
-        <v>1508881.142392117</v>
+        <v>1497503.768858282</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -24337,7 +24337,7 @@
         <v>45869</v>
       </c>
       <c r="B55">
-        <v>1505364.122021733</v>
+        <v>1493986.320460237</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -24345,7 +24345,7 @@
         <v>45870</v>
       </c>
       <c r="B56">
-        <v>1502336.851097612</v>
+        <v>1490959.538728738</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -24353,7 +24353,7 @@
         <v>45873</v>
       </c>
       <c r="B57">
-        <v>1510183.922755687</v>
+        <v>1498806.009650609</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -24361,7 +24361,7 @@
         <v>45874</v>
       </c>
       <c r="B58">
-        <v>1509886.852630879</v>
+        <v>1498508.771233282</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -24369,7 +24369,7 @@
         <v>45875</v>
       </c>
       <c r="B59">
-        <v>1512663.073419059</v>
+        <v>1501284.994745236</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -24377,7 +24377,7 @@
         <v>45876</v>
       </c>
       <c r="B60">
-        <v>1514713.526210101</v>
+        <v>1503335.537292832</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -24385,7 +24385,7 @@
         <v>45877</v>
       </c>
       <c r="B61">
-        <v>1515545.400258482</v>
+        <v>1504167.311483528</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -24393,7 +24393,7 @@
         <v>45880</v>
       </c>
       <c r="B62">
-        <v>1512607.105444743</v>
+        <v>1501228.964699782</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -24401,7 +24401,7 @@
         <v>45881</v>
       </c>
       <c r="B63">
-        <v>1525190.229752296</v>
+        <v>1513813.73513428</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -24409,7 +24409,7 @@
         <v>45882</v>
       </c>
       <c r="B64">
-        <v>1536383.456702683</v>
+        <v>1525008.039078961</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -24417,7 +24417,7 @@
         <v>45883</v>
       </c>
       <c r="B65">
-        <v>1525753.588706144</v>
+        <v>1514376.949552855</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -24425,7 +24425,7 @@
         <v>45884</v>
       </c>
       <c r="B66">
-        <v>1528159.531709514</v>
+        <v>1516782.845172878</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -24433,7 +24433,7 @@
         <v>45887</v>
       </c>
       <c r="B67">
-        <v>1527406.397653332</v>
+        <v>1516029.724539743</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -24441,7 +24441,7 @@
         <v>45888</v>
       </c>
       <c r="B68">
-        <v>1522592.7535748</v>
+        <v>1511216.007887808</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -24449,7 +24449,7 @@
         <v>45889</v>
       </c>
       <c r="B69">
-        <v>1522678.384991582</v>
+        <v>1511301.555789805</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -24457,7 +24457,7 @@
         <v>45890</v>
       </c>
       <c r="B70">
-        <v>1516239.68215742</v>
+        <v>1504862.654609832</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -24465,7 +24465,7 @@
         <v>45891</v>
       </c>
       <c r="B71">
-        <v>1537188.854496558</v>
+        <v>1525811.883218108</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -24473,7 +24473,7 @@
         <v>45894</v>
       </c>
       <c r="B72">
-        <v>1527760.872203784</v>
+        <v>1516383.909903698</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -24481,7 +24481,7 @@
         <v>45895</v>
       </c>
       <c r="B73">
-        <v>1531222.046201163</v>
+        <v>1519845.161627616</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -24489,7 +24489,7 @@
         <v>45896</v>
       </c>
       <c r="B74">
-        <v>1530557.870036136</v>
+        <v>1519180.869158247</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -24497,7 +24497,7 @@
         <v>45897</v>
       </c>
       <c r="B75">
-        <v>1538014.442663789</v>
+        <v>1526637.552266011</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -24505,7 +24505,7 @@
         <v>45898</v>
       </c>
       <c r="B76">
-        <v>1537225.883026081</v>
+        <v>1525849.680467402</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -24513,7 +24513,7 @@
         <v>45901</v>
       </c>
       <c r="B77">
-        <v>1537208.404492826</v>
+        <v>1525832.194636981</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -24521,7 +24521,7 @@
         <v>45902</v>
       </c>
       <c r="B78">
-        <v>1531949.14611996</v>
+        <v>1520571.827946947</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -24529,7 +24529,7 @@
         <v>45903</v>
       </c>
       <c r="B79">
-        <v>1540244.91573486</v>
+        <v>1528868.020507671</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -24537,7 +24537,7 @@
         <v>45904</v>
       </c>
       <c r="B80">
-        <v>1544247.726172321</v>
+        <v>1532870.797955559</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -24545,7 +24545,7 @@
         <v>45905</v>
       </c>
       <c r="B81">
-        <v>1554783.522750359</v>
+        <v>1543406.997370788</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -24553,7 +24553,7 @@
         <v>45908</v>
       </c>
       <c r="B82">
-        <v>1562400.228995592</v>
+        <v>1551023.844128225</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -24561,7 +24561,7 @@
         <v>45909</v>
       </c>
       <c r="B83">
-        <v>1558633.733729265</v>
+        <v>1547257.421584345</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -24569,7 +24569,7 @@
         <v>45910</v>
       </c>
       <c r="B84">
-        <v>1566872.187738622</v>
+        <v>1555495.87662424</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -24577,7 +24577,7 @@
         <v>45911</v>
       </c>
       <c r="B85">
-        <v>1582356.461541917</v>
+        <v>1570980.179306903</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -24585,7 +24585,7 @@
         <v>45912</v>
       </c>
       <c r="B86">
-        <v>1577036.446918947</v>
+        <v>1565660.141639695</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -24593,7 +24593,7 @@
         <v>45915</v>
       </c>
       <c r="B87">
-        <v>1594915.324983053</v>
+        <v>1583539.1662634</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -24601,7 +24601,7 @@
         <v>45916</v>
       </c>
       <c r="B88">
-        <v>1598226.35584111</v>
+        <v>1586850.415424882</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -24609,7 +24609,7 @@
         <v>45917</v>
       </c>
       <c r="B89">
-        <v>1591054.11017885</v>
+        <v>1579678.024198088</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -24617,7 +24617,7 @@
         <v>45918</v>
       </c>
       <c r="B90">
-        <v>1583316.547036933</v>
+        <v>1571940.45111638</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -24625,7 +24625,7 @@
         <v>45919</v>
       </c>
       <c r="B91">
-        <v>1583456.545705235</v>
+        <v>1572080.416037514</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -24633,7 +24633,7 @@
         <v>45922</v>
       </c>
       <c r="B92">
-        <v>1595100.477552664</v>
+        <v>1583724.5909845</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -24641,7 +24641,7 @@
         <v>45923</v>
       </c>
       <c r="B93">
-        <v>1597111.091984306</v>
+        <v>1585735.21034996</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -24649,7 +24649,7 @@
         <v>45924</v>
       </c>
       <c r="B94">
-        <v>1586421.930726261</v>
+        <v>1575046.025218158</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -24657,7 +24657,7 @@
         <v>45925</v>
       </c>
       <c r="B95">
-        <v>1576405.447711954</v>
+        <v>1565029.514673457</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -24665,7 +24665,7 @@
         <v>45926</v>
       </c>
       <c r="B96">
-        <v>1582089.341647386</v>
+        <v>1570713.442519763</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -24673,7 +24673,7 @@
         <v>45929</v>
       </c>
       <c r="B97">
-        <v>1590849.558876955</v>
+        <v>1579473.699560636</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -24681,7 +24681,7 @@
         <v>45930</v>
       </c>
       <c r="B98">
-        <v>1594867.043132049</v>
+        <v>1583491.213701776</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -24689,7 +24689,7 @@
         <v>45931</v>
       </c>
       <c r="B99">
-        <v>1600306.215468304</v>
+        <v>1588930.465032704</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -24697,7 +24697,7 @@
         <v>45932</v>
       </c>
       <c r="B100">
-        <v>1600656.786816958</v>
+        <v>1589281.006376688</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -24705,7 +24705,7 @@
         <v>45933</v>
       </c>
       <c r="B101">
-        <v>1607904.516701709</v>
+        <v>1596528.770264261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
learning pysystemtrade. Stopped working on ETF Carry strategy and start working on Dynamic Optimization.
</commit_message>
<xml_diff>
--- a/perplexity_examples/cash_weights_time_series.xlsx
+++ b/perplexity_examples/cash_weights_time_series.xlsx
@@ -614,28 +614,28 @@
         <v>0.06747301079568173</v>
       </c>
       <c r="C2">
-        <v>0.6875927329392475</v>
+        <v>0.6927218017618419</v>
       </c>
       <c r="D2">
-        <v>0.1091519624791499</v>
+        <v>0.1099661769128651</v>
       </c>
       <c r="E2">
         <v>0.12</v>
       </c>
       <c r="F2">
-        <v>1.099384722678919</v>
+        <v>1.091244629656312</v>
       </c>
       <c r="G2">
-        <v>0.07417879726192224</v>
+        <v>0.07362956067753006</v>
       </c>
       <c r="H2">
-        <v>1.099384722678919</v>
+        <v>1.091244629656312</v>
       </c>
       <c r="I2">
-        <v>0.09938472267891862</v>
+        <v>0.09124462965631208</v>
       </c>
       <c r="J2">
-        <v>0.00670578646624051</v>
+        <v>0.006156549881848328</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -646,28 +646,28 @@
         <v>0.08506597361055578</v>
       </c>
       <c r="C3">
-        <v>0.4731132442859182</v>
+        <v>0.4678665293461374</v>
       </c>
       <c r="D3">
-        <v>0.0751043991810894</v>
+        <v>0.07427150900524697</v>
       </c>
       <c r="E3">
         <v>0.12</v>
       </c>
       <c r="F3">
-        <v>1.597775913374391</v>
+        <v>1.615693576274618</v>
       </c>
       <c r="G3">
-        <v>0.1359163636826876</v>
+        <v>0.1374405471221212</v>
       </c>
       <c r="H3">
-        <v>1.597775913374391</v>
+        <v>1.615693576274618</v>
       </c>
       <c r="I3">
-        <v>0.5977759133743914</v>
+        <v>0.6156935762746183</v>
       </c>
       <c r="J3">
-        <v>0.05085039007213187</v>
+        <v>0.05237457351156539</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -678,28 +678,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C4">
-        <v>0.2225057821642802</v>
+        <v>0.22388943747094</v>
       </c>
       <c r="D4">
-        <v>0.0353216978928358</v>
+        <v>0.0355413463633352</v>
       </c>
       <c r="E4">
         <v>0.12</v>
       </c>
       <c r="F4">
-        <v>3.397345177575375</v>
+        <v>3.376349302394272</v>
       </c>
       <c r="G4">
-        <v>0.01867792730574227</v>
+        <v>0.01856249616470261</v>
       </c>
       <c r="H4">
-        <v>3.397345177575375</v>
+        <v>3.376349302394272</v>
       </c>
       <c r="I4">
-        <v>2.397345177575375</v>
+        <v>2.376349302394272</v>
       </c>
       <c r="J4">
-        <v>0.01318012642609413</v>
+        <v>0.01306469528505447</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -710,28 +710,28 @@
         <v>0.0505797680927629</v>
       </c>
       <c r="C5">
-        <v>0.3273856119345384</v>
+        <v>0.3093800316320641</v>
       </c>
       <c r="D5">
-        <v>0.05197085471996929</v>
+        <v>0.04911255745846429</v>
       </c>
       <c r="E5">
         <v>0.12</v>
       </c>
       <c r="F5">
-        <v>2.308986462635397</v>
+        <v>2.443366955619996</v>
       </c>
       <c r="G5">
-        <v>0.1167879998094273</v>
+        <v>0.1235849339807795</v>
       </c>
       <c r="H5">
-        <v>2.308986462635397</v>
+        <v>2.443366955619996</v>
       </c>
       <c r="I5">
-        <v>1.308986462635397</v>
+        <v>1.443366955619996</v>
       </c>
       <c r="J5">
-        <v>0.0662082317166644</v>
+        <v>0.07300516588801659</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -742,28 +742,28 @@
         <v>0.01859256297481008</v>
       </c>
       <c r="C6">
-        <v>0.3455609289392764</v>
+        <v>0.3350601889271543</v>
       </c>
       <c r="D6">
-        <v>0.05485609684762731</v>
+        <v>0.05318915604837407</v>
       </c>
       <c r="E6">
         <v>0.12</v>
       </c>
       <c r="F6">
-        <v>2.187541711786779</v>
+        <v>2.256098966692822</v>
       </c>
       <c r="G6">
-        <v>0.04067200703641953</v>
+        <v>0.04194666211564024</v>
       </c>
       <c r="H6">
-        <v>2.187541711786779</v>
+        <v>2.256098966692822</v>
       </c>
       <c r="I6">
-        <v>1.187541711786779</v>
+        <v>1.256098966692822</v>
       </c>
       <c r="J6">
-        <v>0.02207944406160945</v>
+        <v>0.02335409914083016</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -774,28 +774,28 @@
         <v>0.01859256297481008</v>
       </c>
       <c r="C7">
-        <v>0.3441034985367146</v>
+        <v>0.323899003955213</v>
       </c>
       <c r="D7">
-        <v>0.05462473694372551</v>
+        <v>0.05141737286202119</v>
       </c>
       <c r="E7">
         <v>0.12</v>
       </c>
       <c r="F7">
-        <v>2.196806917782033</v>
+        <v>2.333841527104481</v>
       </c>
       <c r="G7">
-        <v>0.04084427096236087</v>
+        <v>0.04339209556591697</v>
       </c>
       <c r="H7">
-        <v>2.196806917782033</v>
+        <v>2.333841527104481</v>
       </c>
       <c r="I7">
-        <v>1.196806917782033</v>
+        <v>1.333841527104481</v>
       </c>
       <c r="J7">
-        <v>0.0222517079875508</v>
+        <v>0.0247995325911069</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -806,28 +806,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C8">
-        <v>1.149830109059218</v>
+        <v>1.221742015995789</v>
       </c>
       <c r="D8">
-        <v>0.182529871112698</v>
+        <v>0.1939455324362133</v>
       </c>
       <c r="E8">
         <v>0.12</v>
       </c>
       <c r="F8">
-        <v>0.6574266407382129</v>
+        <v>0.6187304161773706</v>
       </c>
       <c r="G8">
-        <v>0.007425950660077774</v>
+        <v>0.006988858159540471</v>
       </c>
       <c r="H8">
-        <v>0.6574266407382129</v>
+        <v>0.6187304161773706</v>
       </c>
       <c r="I8">
-        <v>-0.3425733592617871</v>
+        <v>-0.3812695838226294</v>
       </c>
       <c r="J8">
-        <v>-0.003869531147199314</v>
+        <v>-0.004306623647736618</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -838,28 +838,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C9">
-        <v>1.044104513543286</v>
+        <v>1.040539139693347</v>
       </c>
       <c r="D9">
-        <v>0.1657464531357363</v>
+        <v>0.1651804675834617</v>
       </c>
       <c r="E9">
         <v>0.12</v>
       </c>
       <c r="F9">
-        <v>0.7239973931854051</v>
+        <v>0.7264781469356654</v>
       </c>
       <c r="G9">
-        <v>0.008177899383241781</v>
+        <v>0.008205920692096179</v>
       </c>
       <c r="H9">
-        <v>0.7239973931854051</v>
+        <v>0.7264781469356654</v>
       </c>
       <c r="I9">
-        <v>-0.2760026068145949</v>
+        <v>-0.2735218530643346</v>
       </c>
       <c r="J9">
-        <v>-0.003117582424035308</v>
+        <v>-0.003089561115180909</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -870,28 +870,28 @@
         <v>0.02249100359856058</v>
       </c>
       <c r="C10">
-        <v>0.5896564487873017</v>
+        <v>0.5929127926897186</v>
       </c>
       <c r="D10">
-        <v>0.09360505934740165</v>
+        <v>0.09412198791634746</v>
       </c>
       <c r="E10">
         <v>0.12</v>
       </c>
       <c r="F10">
-        <v>1.281981987262433</v>
+        <v>1.274941197657789</v>
       </c>
       <c r="G10">
-        <v>0.02883306148880923</v>
+        <v>0.02867470706447446</v>
       </c>
       <c r="H10">
-        <v>1.281981987262433</v>
+        <v>1.274941197657789</v>
       </c>
       <c r="I10">
-        <v>0.2819819872624334</v>
+        <v>0.2749411976577891</v>
       </c>
       <c r="J10">
-        <v>0.006342057890248651</v>
+        <v>0.00618370346591389</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -902,28 +902,28 @@
         <v>0.04498200719712115</v>
       </c>
       <c r="C11">
-        <v>0.8481068789469011</v>
+        <v>0.8679816038577943</v>
       </c>
       <c r="D11">
-        <v>0.1346327932137997</v>
+        <v>0.1377878079832023</v>
       </c>
       <c r="E11">
         <v>0.12</v>
       </c>
       <c r="F11">
-        <v>0.8913133058855689</v>
+        <v>0.8709043402056962</v>
       </c>
       <c r="G11">
-        <v>0.0400930615402345</v>
+        <v>0.03917502529913667</v>
       </c>
       <c r="H11">
-        <v>0.8913133058855689</v>
+        <v>0.8709043402056962</v>
       </c>
       <c r="I11">
-        <v>-0.1086866941144311</v>
+        <v>-0.1290956597943038</v>
       </c>
       <c r="J11">
-        <v>-0.004888945656886648</v>
+        <v>-0.005806981897984481</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -934,28 +934,28 @@
         <v>0.007297081167532987</v>
       </c>
       <c r="C12">
-        <v>0.2755045394670109</v>
+        <v>0.2739170049851765</v>
       </c>
       <c r="D12">
-        <v>0.04373498978994543</v>
+        <v>0.043482976503745</v>
       </c>
       <c r="E12">
         <v>0.12</v>
       </c>
       <c r="F12">
-        <v>2.743798514103865</v>
+        <v>2.759700684005956</v>
       </c>
       <c r="G12">
-        <v>0.02002172046477231</v>
+        <v>0.02013775988928776</v>
       </c>
       <c r="H12">
-        <v>2.743798514103865</v>
+        <v>2.759700684005956</v>
       </c>
       <c r="I12">
-        <v>1.743798514103865</v>
+        <v>1.759700684005956</v>
       </c>
       <c r="J12">
-        <v>0.01272463929723932</v>
+        <v>0.01284067872175478</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -966,28 +966,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C13">
-        <v>0.2194362678391605</v>
+        <v>0.2028519346467345</v>
       </c>
       <c r="D13">
-        <v>0.03483442759983477</v>
+        <v>0.03220174632261519</v>
       </c>
       <c r="E13">
         <v>0.12</v>
       </c>
       <c r="F13">
-        <v>3.444867858272751</v>
+        <v>3.726505972619391</v>
       </c>
       <c r="G13">
-        <v>0.01893919754148354</v>
+        <v>0.02048758781428094</v>
       </c>
       <c r="H13">
-        <v>3.444867858272751</v>
+        <v>3.726505972619391</v>
       </c>
       <c r="I13">
-        <v>2.444867858272751</v>
+        <v>2.726505972619391</v>
       </c>
       <c r="J13">
-        <v>0.0134413966618354</v>
+        <v>0.0149897869346328</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -998,28 +998,28 @@
         <v>0.09996001599360257</v>
       </c>
       <c r="C14">
-        <v>0.6720362513692257</v>
+        <v>0.7374920779455986</v>
       </c>
       <c r="D14">
-        <v>0.1066824475885837</v>
+        <v>0.117073237927459</v>
       </c>
       <c r="E14">
         <v>0.12</v>
       </c>
       <c r="F14">
-        <v>1.124833585209583</v>
+        <v>1.024999411687533</v>
       </c>
       <c r="G14">
-        <v>0.1124383831676912</v>
+        <v>0.102458957585719</v>
       </c>
       <c r="H14">
-        <v>1.124833585209583</v>
+        <v>1.024999411687533</v>
       </c>
       <c r="I14">
-        <v>0.1248335852095825</v>
+        <v>0.0249994116875325</v>
       </c>
       <c r="J14">
-        <v>0.01247836717408862</v>
+        <v>0.002498941592116402</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1030,28 +1030,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C15">
-        <v>0.5204775825744208</v>
+        <v>0.4899100306438611</v>
       </c>
       <c r="D15">
-        <v>0.08262325478856015</v>
+        <v>0.07777080635278136</v>
       </c>
       <c r="E15">
         <v>0.12</v>
       </c>
       <c r="F15">
-        <v>1.452375609107752</v>
+        <v>1.542995445561667</v>
       </c>
       <c r="G15">
-        <v>0.0079848719013321</v>
+        <v>0.008483081717902007</v>
       </c>
       <c r="H15">
-        <v>1.452375609107752</v>
+        <v>1.542995445561667</v>
       </c>
       <c r="I15">
-        <v>0.4523756091077515</v>
+        <v>0.542995445561667</v>
       </c>
       <c r="J15">
-        <v>0.00248707102168396</v>
+        <v>0.002985280838253866</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1062,28 +1062,28 @@
         <v>0.04498200719712115</v>
       </c>
       <c r="C16">
-        <v>0.6010991543786579</v>
+        <v>0.5907154947310518</v>
       </c>
       <c r="D16">
-        <v>0.09542153254662906</v>
+        <v>0.09377317767905093</v>
       </c>
       <c r="E16">
         <v>0.12</v>
       </c>
       <c r="F16">
-        <v>1.257577789807141</v>
+        <v>1.279683625638808</v>
       </c>
       <c r="G16">
-        <v>0.05656837319204455</v>
+        <v>0.05756273805852293</v>
       </c>
       <c r="H16">
-        <v>1.257577789807141</v>
+        <v>1.279683625638808</v>
       </c>
       <c r="I16">
-        <v>0.2575777898071414</v>
+        <v>0.2796836256388076</v>
       </c>
       <c r="J16">
-        <v>0.01158636599492339</v>
+        <v>0.01258073086140178</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1094,28 +1094,28 @@
         <v>0.06377449020391843</v>
       </c>
       <c r="C17">
-        <v>0.3048640068295793</v>
+        <v>0.2958283399997339</v>
       </c>
       <c r="D17">
-        <v>0.04839566074594583</v>
+        <v>0.04696129310426145</v>
       </c>
       <c r="E17">
         <v>0.12</v>
       </c>
       <c r="F17">
-        <v>2.479561145573419</v>
+        <v>2.55529590579163</v>
       </c>
       <c r="G17">
-        <v>0.1581327479883888</v>
+        <v>0.1629626937120212</v>
       </c>
       <c r="H17">
-        <v>2.479561145573419</v>
+        <v>2.55529590579163</v>
       </c>
       <c r="I17">
-        <v>1.479561145573419</v>
+        <v>1.55529590579163</v>
       </c>
       <c r="J17">
-        <v>0.09435825778447035</v>
+        <v>0.09918820350810273</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1126,28 +1126,28 @@
         <v>0.03378648540583766</v>
       </c>
       <c r="C18">
-        <v>0.9309805005368549</v>
+        <v>0.912266961315544</v>
       </c>
       <c r="D18">
-        <v>0.1477885727922572</v>
+        <v>0.1448178905364906</v>
       </c>
       <c r="E18">
         <v>0.12</v>
       </c>
       <c r="F18">
-        <v>0.8119707615600369</v>
+        <v>0.8286269020730065</v>
       </c>
       <c r="G18">
-        <v>0.02743363828541508</v>
+        <v>0.02799639073377411</v>
       </c>
       <c r="H18">
-        <v>0.8119707615600369</v>
+        <v>0.8286269020730065</v>
       </c>
       <c r="I18">
-        <v>-0.1880292384399631</v>
+        <v>-0.1713730979269935</v>
       </c>
       <c r="J18">
-        <v>-0.006352847120422583</v>
+        <v>-0.005790094672063553</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1158,28 +1158,28 @@
         <v>0.0899640143942423</v>
       </c>
       <c r="C19">
-        <v>0.5637687130383457</v>
+        <v>0.5850247960208312</v>
       </c>
       <c r="D19">
-        <v>0.08949550869950401</v>
+        <v>0.09286980726464454</v>
       </c>
       <c r="E19">
         <v>0.12</v>
       </c>
       <c r="F19">
-        <v>1.340849409582327</v>
+        <v>1.292131463760277</v>
       </c>
       <c r="G19">
-        <v>0.1206281955841758</v>
+        <v>0.116245333604983</v>
       </c>
       <c r="H19">
-        <v>1.340849409582327</v>
+        <v>1.292131463760277</v>
       </c>
       <c r="I19">
-        <v>0.3408494095823273</v>
+        <v>0.2921314637602774</v>
       </c>
       <c r="J19">
-        <v>0.03066418118993348</v>
+        <v>0.02628131921074067</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1190,28 +1190,28 @@
         <v>0.01129548180727709</v>
       </c>
       <c r="C20">
-        <v>1.203238540997612</v>
+        <v>1.200236433410926</v>
       </c>
       <c r="D20">
-        <v>0.1910081968420727</v>
+        <v>0.1905316270370667</v>
       </c>
       <c r="E20">
         <v>0.12</v>
       </c>
       <c r="F20">
-        <v>0.6282452899087735</v>
+        <v>0.6298166969237855</v>
       </c>
       <c r="G20">
-        <v>0.007096333242672071</v>
+        <v>0.007114083042021967</v>
       </c>
       <c r="H20">
-        <v>0.6282452899087735</v>
+        <v>0.6298166969237855</v>
       </c>
       <c r="I20">
-        <v>-0.3717547100912265</v>
+        <v>-0.3701833030762145</v>
       </c>
       <c r="J20">
-        <v>-0.004199148564605017</v>
+        <v>-0.004181398765255122</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1222,28 +1222,28 @@
         <v>0.06377449020391843</v>
       </c>
       <c r="C21">
-        <v>0.4767687285570399</v>
+        <v>0.4541639742296063</v>
       </c>
       <c r="D21">
-        <v>0.07568468931926318</v>
+        <v>0.07209629581537716</v>
       </c>
       <c r="E21">
         <v>0.12</v>
       </c>
       <c r="F21">
-        <v>1.585525435584469</v>
+        <v>1.66444057413565</v>
       </c>
       <c r="G21">
-        <v>0.1011160763597452</v>
+        <v>0.1061488490902184</v>
       </c>
       <c r="H21">
-        <v>1.585525435584469</v>
+        <v>1.66444057413565</v>
       </c>
       <c r="I21">
-        <v>0.5855254355844692</v>
+        <v>0.6644405741356496</v>
       </c>
       <c r="J21">
-        <v>0.03734158615582681</v>
+        <v>0.04237435888629992</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1254,28 +1254,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C22">
-        <v>0.09491058452950714</v>
+        <v>0.09674696391196448</v>
       </c>
       <c r="D22">
-        <v>0.01506658820717101</v>
+        <v>0.01535810439669592</v>
       </c>
       <c r="E22">
         <v>0.12</v>
       </c>
       <c r="F22">
-        <v>7.964643245700806</v>
+        <v>7.813464272701278</v>
       </c>
       <c r="G22">
-        <v>0.07244927382634681</v>
+        <v>0.07107409524348425</v>
       </c>
       <c r="H22">
-        <v>7.964643245700806</v>
+        <v>7.813464272701278</v>
       </c>
       <c r="I22">
-        <v>6.964643245700806</v>
+        <v>6.813464272701278</v>
       </c>
       <c r="J22">
-        <v>0.06335291237092897</v>
+        <v>0.06197773378806642</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1286,28 +1286,28 @@
         <v>0.01009596161535386</v>
       </c>
       <c r="C23">
-        <v>0.2305035920630537</v>
+        <v>0.21620725284203</v>
       </c>
       <c r="D23">
-        <v>0.0365913108543553</v>
+        <v>0.03432183736010846</v>
       </c>
       <c r="E23">
         <v>0.12</v>
       </c>
       <c r="F23">
-        <v>3.279467097465761</v>
+        <v>3.496316317245691</v>
       </c>
       <c r="G23">
-        <v>0.03310937393483026</v>
+        <v>0.03529867533404786</v>
       </c>
       <c r="H23">
-        <v>3.279467097465761</v>
+        <v>3.496316317245691</v>
       </c>
       <c r="I23">
-        <v>2.279467097465761</v>
+        <v>2.496316317245691</v>
       </c>
       <c r="J23">
-        <v>0.0230134123194764</v>
+        <v>0.025202713718694</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1318,28 +1318,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C24">
-        <v>0.2204874680312308</v>
+        <v>0.2153786668053592</v>
       </c>
       <c r="D24">
-        <v>0.03500130045701645</v>
+        <v>0.03419030340453737</v>
       </c>
       <c r="E24">
         <v>0.12</v>
       </c>
       <c r="F24">
-        <v>3.428444041596874</v>
+        <v>3.509767040677238</v>
       </c>
       <c r="G24">
-        <v>0.03118636623203874</v>
+        <v>0.03192610962631234</v>
       </c>
       <c r="H24">
-        <v>3.428444041596874</v>
+        <v>3.509767040677238</v>
       </c>
       <c r="I24">
-        <v>2.428444041596874</v>
+        <v>2.509767040677238</v>
       </c>
       <c r="J24">
-        <v>0.02209000477662091</v>
+        <v>0.02282974817089451</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1350,28 +1350,28 @@
         <v>0.005497800879648141</v>
       </c>
       <c r="C25">
-        <v>0.2047355906627088</v>
+        <v>0.1905957831399994</v>
       </c>
       <c r="D25">
-        <v>0.03250076744504671</v>
+        <v>0.03025614258756215</v>
       </c>
       <c r="E25">
         <v>0.12</v>
       </c>
       <c r="F25">
-        <v>3.69222050534344</v>
+        <v>3.966136782067196</v>
       </c>
       <c r="G25">
-        <v>0.02029909314213206</v>
+        <v>0.02180503028925388</v>
       </c>
       <c r="H25">
-        <v>3.69222050534344</v>
+        <v>3.966136782067196</v>
       </c>
       <c r="I25">
-        <v>2.69222050534344</v>
+        <v>2.966136782067196</v>
       </c>
       <c r="J25">
-        <v>0.01480129226248392</v>
+        <v>0.01630722940960574</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1382,28 +1382,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C26">
-        <v>0.08915061329486798</v>
+        <v>0.08789486232491861</v>
       </c>
       <c r="D26">
-        <v>0.01415222112042656</v>
+        <v>0.01395287683391971</v>
       </c>
       <c r="E26">
         <v>0.12</v>
       </c>
       <c r="F26">
-        <v>8.479234388642956</v>
+        <v>8.600376927880403</v>
       </c>
       <c r="G26">
-        <v>0.07713018086430519</v>
+        <v>0.07823213718883615</v>
       </c>
       <c r="H26">
-        <v>8.479234388642956</v>
+        <v>8.600376927880403</v>
       </c>
       <c r="I26">
-        <v>7.479234388642956</v>
+        <v>7.600376927880403</v>
       </c>
       <c r="J26">
-        <v>0.06803381940888735</v>
+        <v>0.06913577573341831</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -1414,28 +1414,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C27">
-        <v>0.6424749624732814</v>
+        <v>0.6029510318830481</v>
       </c>
       <c r="D27">
-        <v>0.1019897384573915</v>
+        <v>0.09571550898673933</v>
       </c>
       <c r="E27">
         <v>0.12</v>
       </c>
       <c r="F27">
-        <v>1.176588957036425</v>
+        <v>1.253715320226998</v>
       </c>
       <c r="G27">
-        <v>0.01070267843765641</v>
+        <v>0.01140424771497969</v>
       </c>
       <c r="H27">
-        <v>1.176588957036425</v>
+        <v>1.253715320226998</v>
       </c>
       <c r="I27">
-        <v>0.176588957036425</v>
+        <v>0.2537153202269979</v>
       </c>
       <c r="J27">
-        <v>0.001606316982238572</v>
+        <v>0.002307886259561857</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -1446,28 +1446,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C28">
-        <v>0.257563036257339</v>
+        <v>0.2522823743623258</v>
       </c>
       <c r="D28">
-        <v>0.04088686445157787</v>
+        <v>0.04004858536365669</v>
       </c>
       <c r="E28">
         <v>0.12</v>
       </c>
       <c r="F28">
-        <v>2.93492791901701</v>
+        <v>2.996360518364218</v>
       </c>
       <c r="G28">
-        <v>0.026697165196976</v>
+        <v>0.02725597832578408</v>
       </c>
       <c r="H28">
-        <v>2.93492791901701</v>
+        <v>2.996360518364218</v>
       </c>
       <c r="I28">
-        <v>1.93492791901701</v>
+        <v>1.996360518364218</v>
       </c>
       <c r="J28">
-        <v>0.01760080374155817</v>
+        <v>0.01815961687036624</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1478,28 +1478,28 @@
         <v>0.009096361455417834</v>
       </c>
       <c r="C29">
-        <v>0.526057906397181</v>
+        <v>0.5126046732296039</v>
       </c>
       <c r="D29">
-        <v>0.08350910373277412</v>
+        <v>0.08137346917530364</v>
       </c>
       <c r="E29">
         <v>0.12</v>
       </c>
       <c r="F29">
-        <v>1.436969080448945</v>
+        <v>1.474682119567532</v>
       </c>
       <c r="G29">
-        <v>0.01307119015602299</v>
+        <v>0.01341424159142797</v>
       </c>
       <c r="H29">
-        <v>1.436969080448945</v>
+        <v>1.474682119567532</v>
       </c>
       <c r="I29">
-        <v>0.436969080448945</v>
+        <v>0.4746821195675319</v>
       </c>
       <c r="J29">
-        <v>0.003974828700605159</v>
+        <v>0.004317880136010137</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1510,28 +1510,28 @@
         <v>0.1124550179928029</v>
       </c>
       <c r="C30">
-        <v>0.6690328016056073</v>
+        <v>0.672466529487568</v>
       </c>
       <c r="D30">
-        <v>0.1062056647195951</v>
+        <v>0.1067507521223273</v>
       </c>
       <c r="E30">
         <v>0.12</v>
       </c>
       <c r="F30">
-        <v>1.129883234729756</v>
+        <v>1.1241138597552</v>
       </c>
       <c r="G30">
-        <v>0.127061039491301</v>
+        <v>0.1264122443247301</v>
       </c>
       <c r="H30">
-        <v>1.129883234729756</v>
+        <v>1.1241138597552</v>
       </c>
       <c r="I30">
-        <v>0.1298832347297556</v>
+        <v>0.1241138597552003</v>
       </c>
       <c r="J30">
-        <v>0.0146060214984981</v>
+        <v>0.01395722633192725</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -1542,28 +1542,28 @@
         <v>0.007297081167532987</v>
       </c>
       <c r="C31">
-        <v>0.2705892621474181</v>
+        <v>0.2760783221537554</v>
       </c>
       <c r="D31">
-        <v>0.0429547137051919</v>
+        <v>0.04382607496768864</v>
       </c>
       <c r="E31">
         <v>0.12</v>
       </c>
       <c r="F31">
-        <v>2.793639851113609</v>
+        <v>2.738095987114328</v>
       </c>
       <c r="G31">
-        <v>0.02038541674643077</v>
+        <v>0.01998010866246961</v>
       </c>
       <c r="H31">
-        <v>2.793639851113609</v>
+        <v>2.738095987114328</v>
       </c>
       <c r="I31">
-        <v>1.793639851113609</v>
+        <v>1.738095987114328</v>
       </c>
       <c r="J31">
-        <v>0.01308833557889778</v>
+        <v>0.01268302749493662</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1574,28 +1574,28 @@
         <v>0.02479008396641344</v>
       </c>
       <c r="C32">
-        <v>0.3148736854601289</v>
+        <v>0.2964540946306327</v>
       </c>
       <c r="D32">
-        <v>0.04998464796755253</v>
+        <v>0.04706062857236777</v>
       </c>
       <c r="E32">
         <v>0.12</v>
       </c>
       <c r="F32">
-        <v>2.400737123884474</v>
+        <v>2.549902192986421</v>
       </c>
       <c r="G32">
-        <v>0.05951447488238201</v>
+        <v>0.06321228947027513</v>
       </c>
       <c r="H32">
-        <v>2.400737123884474</v>
+        <v>2.549902192986421</v>
       </c>
       <c r="I32">
-        <v>1.400737123884474</v>
+        <v>1.549902192986421</v>
       </c>
       <c r="J32">
-        <v>0.03472439091596857</v>
+        <v>0.03842220550386169</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1606,28 +1606,28 @@
         <v>0.0235905637744902</v>
       </c>
       <c r="C33">
-        <v>0.5149152336289413</v>
+        <v>0.4984020392457882</v>
       </c>
       <c r="D33">
-        <v>0.0817402592676541</v>
+        <v>0.07911887092630859</v>
       </c>
       <c r="E33">
         <v>0.12</v>
       </c>
       <c r="F33">
-        <v>1.468064832129617</v>
+        <v>1.516705162688281</v>
       </c>
       <c r="G33">
-        <v>0.03463247704743998</v>
+        <v>0.03577992986749644</v>
       </c>
       <c r="H33">
-        <v>1.468064832129617</v>
+        <v>1.516705162688281</v>
       </c>
       <c r="I33">
-        <v>0.468064832129617</v>
+        <v>0.5167051626882813</v>
       </c>
       <c r="J33">
-        <v>0.01104191327294978</v>
+        <v>0.01218936609300623</v>
       </c>
     </row>
   </sheetData>
@@ -23913,7 +23913,7 @@
         <v>45797</v>
       </c>
       <c r="B2">
-        <v>1302231.637486183</v>
+        <v>1071321.262947129</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -23921,7 +23921,7 @@
         <v>45798</v>
       </c>
       <c r="B3">
-        <v>1294256.048624723</v>
+        <v>1067255.712469967</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -23929,7 +23929,7 @@
         <v>45799</v>
       </c>
       <c r="B4">
-        <v>1294491.453335582</v>
+        <v>1067332.590108231</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -23937,7 +23937,7 @@
         <v>45800</v>
       </c>
       <c r="B5">
-        <v>1300198.047750686</v>
+        <v>1070187.857977456</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -23945,7 +23945,7 @@
         <v>45803</v>
       </c>
       <c r="B6">
-        <v>1300176.860558796</v>
+        <v>1070179.246690404</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -23953,7 +23953,7 @@
         <v>45804</v>
       </c>
       <c r="B7">
-        <v>1304602.240558795</v>
+        <v>1072808.553541187</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -23961,7 +23961,7 @@
         <v>45805</v>
       </c>
       <c r="B8">
-        <v>1299000.503916627</v>
+        <v>1069892.658331321</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -23969,7 +23969,7 @@
         <v>45806</v>
       </c>
       <c r="B9">
-        <v>1306364.954468365</v>
+        <v>1073667.826333973</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -23977,7 +23977,7 @@
         <v>45807</v>
       </c>
       <c r="B10">
-        <v>1305894.848264134</v>
+        <v>1073252.827617459</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -23985,7 +23985,7 @@
         <v>45810</v>
       </c>
       <c r="B11">
-        <v>1317133.774641945</v>
+        <v>1079599.620790126</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -23993,7 +23993,7 @@
         <v>45811</v>
       </c>
       <c r="B12">
-        <v>1312830.077192187</v>
+        <v>1077117.302129616</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -24001,7 +24001,7 @@
         <v>45812</v>
       </c>
       <c r="B13">
-        <v>1321321.742811051</v>
+        <v>1081600.289364395</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -24009,7 +24009,7 @@
         <v>45813</v>
       </c>
       <c r="B14">
-        <v>1318938.822018602</v>
+        <v>1080570.131782702</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -24017,7 +24017,7 @@
         <v>45814</v>
       </c>
       <c r="B15">
-        <v>1315609.131506227</v>
+        <v>1078774.203113831</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -24025,7 +24025,7 @@
         <v>45817</v>
       </c>
       <c r="B16">
-        <v>1320844.719758587</v>
+        <v>1081715.666316274</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -24033,7 +24033,7 @@
         <v>45818</v>
       </c>
       <c r="B17">
-        <v>1326501.845793016</v>
+        <v>1084957.462322686</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -24041,7 +24041,7 @@
         <v>45819</v>
       </c>
       <c r="B18">
-        <v>1329882.934304034</v>
+        <v>1087238.382864546</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -24049,7 +24049,7 @@
         <v>45820</v>
       </c>
       <c r="B19">
-        <v>1341810.911875755</v>
+        <v>1094416.836052082</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -24057,7 +24057,7 @@
         <v>45821</v>
       </c>
       <c r="B20">
-        <v>1326018.558239879</v>
+        <v>1085512.429807461</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -24065,7 +24065,7 @@
         <v>45824</v>
       </c>
       <c r="B21">
-        <v>1331718.118755926</v>
+        <v>1088949.971782728</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -24073,7 +24073,7 @@
         <v>45825</v>
       </c>
       <c r="B22">
-        <v>1319108.843507347</v>
+        <v>1080911.933346293</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -24081,7 +24081,7 @@
         <v>45826</v>
       </c>
       <c r="B23">
-        <v>1318983.132381273</v>
+        <v>1080903.706075516</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -24089,7 +24089,7 @@
         <v>45827</v>
       </c>
       <c r="B24">
-        <v>1318962.380956756</v>
+        <v>1080895.775994994</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -24097,7 +24097,7 @@
         <v>45828</v>
       </c>
       <c r="B25">
-        <v>1317509.941860961</v>
+        <v>1080173.407969345</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -24105,7 +24105,7 @@
         <v>45831</v>
       </c>
       <c r="B26">
-        <v>1324545.248587131</v>
+        <v>1084959.520662883</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -24113,7 +24113,7 @@
         <v>45832</v>
       </c>
       <c r="B27">
-        <v>1333528.424556571</v>
+        <v>1092275.410782654</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -24121,7 +24121,7 @@
         <v>45833</v>
       </c>
       <c r="B28">
-        <v>1330826.341238698</v>
+        <v>1090471.988587544</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -24129,7 +24129,7 @@
         <v>45834</v>
       </c>
       <c r="B29">
-        <v>1341562.186393025</v>
+        <v>1096520.057020731</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -24137,7 +24137,7 @@
         <v>45835</v>
       </c>
       <c r="B30">
-        <v>1338893.336495143</v>
+        <v>1094768.300095204</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -24145,7 +24145,7 @@
         <v>45838</v>
       </c>
       <c r="B31">
-        <v>1352108.080294607</v>
+        <v>1102412.217309367</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -24153,7 +24153,7 @@
         <v>45839</v>
       </c>
       <c r="B32">
-        <v>1354588.151332423</v>
+        <v>1103923.322779096</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -24161,7 +24161,7 @@
         <v>45840</v>
       </c>
       <c r="B33">
-        <v>1354489.951310195</v>
+        <v>1103631.980836717</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -24169,7 +24169,7 @@
         <v>45841</v>
       </c>
       <c r="B34">
-        <v>1357359.1957966</v>
+        <v>1105320.952060815</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -24177,7 +24177,7 @@
         <v>45842</v>
       </c>
       <c r="B35">
-        <v>1357347.772678532</v>
+        <v>1105316.203016737</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -24185,7 +24185,7 @@
         <v>45845</v>
       </c>
       <c r="B36">
-        <v>1337255.601263132</v>
+        <v>1093387.298678443</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -24193,7 +24193,7 @@
         <v>45846</v>
       </c>
       <c r="B37">
-        <v>1337384.827692452</v>
+        <v>1093421.542390413</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -24201,7 +24201,7 @@
         <v>45847</v>
       </c>
       <c r="B38">
-        <v>1345698.606152554</v>
+        <v>1099146.871938087</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -24209,7 +24209,7 @@
         <v>45848</v>
       </c>
       <c r="B39">
-        <v>1345877.48976604</v>
+        <v>1098961.352401046</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -24217,7 +24217,7 @@
         <v>45849</v>
       </c>
       <c r="B40">
-        <v>1337930.617069695</v>
+        <v>1093137.643426792</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -24225,7 +24225,7 @@
         <v>45852</v>
       </c>
       <c r="B41">
-        <v>1338679.193696191</v>
+        <v>1093224.270837745</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -24233,7 +24233,7 @@
         <v>45853</v>
       </c>
       <c r="B42">
-        <v>1331867.126668832</v>
+        <v>1088064.037359752</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -24241,7 +24241,7 @@
         <v>45854</v>
       </c>
       <c r="B43">
-        <v>1336044.53934955</v>
+        <v>1091431.759411235</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -24249,7 +24249,7 @@
         <v>45855</v>
       </c>
       <c r="B44">
-        <v>1339026.870758226</v>
+        <v>1092781.133278977</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -24257,7 +24257,7 @@
         <v>45856</v>
       </c>
       <c r="B45">
-        <v>1340337.346016591</v>
+        <v>1094179.019206204</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -24265,7 +24265,7 @@
         <v>45859</v>
       </c>
       <c r="B46">
-        <v>1343605.552852619</v>
+        <v>1097094.242851876</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -24273,7 +24273,7 @@
         <v>45860</v>
       </c>
       <c r="B47">
-        <v>1347774.011370222</v>
+        <v>1100534.933238055</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -24281,7 +24281,7 @@
         <v>45861</v>
       </c>
       <c r="B48">
-        <v>1352038.346467231</v>
+        <v>1103071.473899088</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -24289,7 +24289,7 @@
         <v>45862</v>
       </c>
       <c r="B49">
-        <v>1346037.140315584</v>
+        <v>1099829.395073792</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -24297,7 +24297,7 @@
         <v>45863</v>
       </c>
       <c r="B50">
-        <v>1344291.568338118</v>
+        <v>1099028.816367388</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -24305,7 +24305,7 @@
         <v>45866</v>
       </c>
       <c r="B51">
-        <v>1330291.099517122</v>
+        <v>1091288.129740219</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -24313,7 +24313,7 @@
         <v>45867</v>
       </c>
       <c r="B52">
-        <v>1333058.888780817</v>
+        <v>1092894.239454186</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -24321,7 +24321,7 @@
         <v>45868</v>
       </c>
       <c r="B53">
-        <v>1324847.072611387</v>
+        <v>1087038.794450637</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -24329,7 +24329,7 @@
         <v>45869</v>
       </c>
       <c r="B54">
-        <v>1321362.054012271</v>
+        <v>1084948.249873193</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -24337,7 +24337,7 @@
         <v>45870</v>
       </c>
       <c r="B55">
-        <v>1317719.601341968</v>
+        <v>1083906.337769954</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -24345,7 +24345,7 @@
         <v>45873</v>
       </c>
       <c r="B56">
-        <v>1325136.397640875</v>
+        <v>1088862.341393209</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -24353,7 +24353,7 @@
         <v>45874</v>
       </c>
       <c r="B57">
-        <v>1324819.542419536</v>
+        <v>1088703.812486806</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -24361,7 +24361,7 @@
         <v>45875</v>
       </c>
       <c r="B58">
-        <v>1326947.206180531</v>
+        <v>1090212.160008949</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -24369,7 +24369,7 @@
         <v>45876</v>
       </c>
       <c r="B59">
-        <v>1328461.48847417</v>
+        <v>1090793.615582749</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -24377,7 +24377,7 @@
         <v>45877</v>
       </c>
       <c r="B60">
-        <v>1329252.416829051</v>
+        <v>1091208.884622353</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -24385,7 +24385,7 @@
         <v>45880</v>
       </c>
       <c r="B61">
-        <v>1326800.80304443</v>
+        <v>1090505.345202737</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -24393,7 +24393,7 @@
         <v>45881</v>
       </c>
       <c r="B62">
-        <v>1338554.487804157</v>
+        <v>1096604.390099911</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -24401,7 +24401,7 @@
         <v>45882</v>
       </c>
       <c r="B63">
-        <v>1349164.409056785</v>
+        <v>1102465.49956004</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -24409,7 +24409,7 @@
         <v>45883</v>
       </c>
       <c r="B64">
-        <v>1338711.634518128</v>
+        <v>1096812.271051308</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -24417,7 +24417,7 @@
         <v>45884</v>
       </c>
       <c r="B65">
-        <v>1341084.3347082</v>
+        <v>1097995.089488088</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -24425,7 +24425,7 @@
         <v>45887</v>
       </c>
       <c r="B66">
-        <v>1340485.721675484</v>
+        <v>1097698.978759607</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -24433,7 +24433,7 @@
         <v>45888</v>
       </c>
       <c r="B67">
-        <v>1335789.119233669</v>
+        <v>1095090.492822394</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -24441,7 +24441,7 @@
         <v>45889</v>
       </c>
       <c r="B68">
-        <v>1335809.842613635</v>
+        <v>1095035.573461256</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -24449,7 +24449,7 @@
         <v>45890</v>
       </c>
       <c r="B69">
-        <v>1329137.044740326</v>
+        <v>1090446.555342607</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -24457,7 +24457,7 @@
         <v>45891</v>
       </c>
       <c r="B70">
-        <v>1350897.429543135</v>
+        <v>1105497.828449043</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -24465,7 +24465,7 @@
         <v>45894</v>
       </c>
       <c r="B71">
-        <v>1340934.33405828</v>
+        <v>1098125.436798573</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -24473,7 +24473,7 @@
         <v>45895</v>
       </c>
       <c r="B72">
-        <v>1344188.725086113</v>
+        <v>1099854.232664261</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -24481,7 +24481,7 @@
         <v>45896</v>
       </c>
       <c r="B73">
-        <v>1343344.993910338</v>
+        <v>1099142.196071909</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -24489,7 +24489,7 @@
         <v>45897</v>
       </c>
       <c r="B74">
-        <v>1350937.021607959</v>
+        <v>1103924.10236806</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -24497,7 +24497,7 @@
         <v>45898</v>
       </c>
       <c r="B75">
-        <v>1349830.213948108</v>
+        <v>1102784.565546267</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -24505,7 +24505,7 @@
         <v>45901</v>
       </c>
       <c r="B76">
-        <v>1349812.764930822</v>
+        <v>1102776.541559421</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -24513,7 +24513,7 @@
         <v>45902</v>
       </c>
       <c r="B77">
-        <v>1344419.95295551</v>
+        <v>1099278.016544894</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -24521,7 +24521,7 @@
         <v>45903</v>
       </c>
       <c r="B78">
-        <v>1352697.011982837</v>
+        <v>1103765.532656464</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -24529,7 +24529,7 @@
         <v>45904</v>
       </c>
       <c r="B79">
-        <v>1356670.231084547</v>
+        <v>1106502.365258695</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -24537,7 +24537,7 @@
         <v>45905</v>
       </c>
       <c r="B80">
-        <v>1367121.054019081</v>
+        <v>1112982.996003478</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -24545,7 +24545,7 @@
         <v>45908</v>
       </c>
       <c r="B81">
-        <v>1374443.405402727</v>
+        <v>1117223.761382654</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -24553,7 +24553,7 @@
         <v>45909</v>
       </c>
       <c r="B82">
-        <v>1371004.432465051</v>
+        <v>1115393.049942943</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -24561,7 +24561,7 @@
         <v>45910</v>
       </c>
       <c r="B83">
-        <v>1379133.735894965</v>
+        <v>1120174.183952861</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -24569,7 +24569,7 @@
         <v>45911</v>
       </c>
       <c r="B84">
-        <v>1393916.85078247</v>
+        <v>1128196.763388322</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -24577,7 +24577,7 @@
         <v>45912</v>
       </c>
       <c r="B85">
-        <v>1388702.446705907</v>
+        <v>1125359.918268155</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -24585,7 +24585,7 @@
         <v>45915</v>
       </c>
       <c r="B86">
-        <v>1406201.447136605</v>
+        <v>1135174.961599917</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -24593,7 +24593,7 @@
         <v>45916</v>
       </c>
       <c r="B87">
-        <v>1409842.805661753</v>
+        <v>1137242.199736953</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -24601,7 +24601,7 @@
         <v>45917</v>
       </c>
       <c r="B88">
-        <v>1402802.342926174</v>
+        <v>1133372.209322663</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -24609,7 +24609,7 @@
         <v>45918</v>
       </c>
       <c r="B89">
-        <v>1394905.629507521</v>
+        <v>1128693.1282147</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -24617,7 +24617,7 @@
         <v>45919</v>
       </c>
       <c r="B90">
-        <v>1394960.54449998</v>
+        <v>1128919.397115531</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -24625,7 +24625,7 @@
         <v>45922</v>
       </c>
       <c r="B91">
-        <v>1406677.742261115</v>
+        <v>1136000.181631615</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -24633,7 +24633,7 @@
         <v>45923</v>
       </c>
       <c r="B92">
-        <v>1409025.267875169</v>
+        <v>1137745.313637962</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -24641,7 +24641,7 @@
         <v>45924</v>
       </c>
       <c r="B93">
-        <v>1397802.497099908</v>
+        <v>1130263.933538392</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -24649,7 +24649,7 @@
         <v>45925</v>
       </c>
       <c r="B94">
-        <v>1387376.26315062</v>
+        <v>1123030.552709038</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -24657,7 +24657,7 @@
         <v>45926</v>
       </c>
       <c r="B95">
-        <v>1393378.547006978</v>
+        <v>1127089.550374356</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -24665,7 +24665,7 @@
         <v>45929</v>
       </c>
       <c r="B96">
-        <v>1402374.412845606</v>
+        <v>1133260.129661014</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -24673,7 +24673,7 @@
         <v>45930</v>
       </c>
       <c r="B97">
-        <v>1406267.765263468</v>
+        <v>1135421.259181015</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -24681,7 +24681,7 @@
         <v>45931</v>
       </c>
       <c r="B98">
-        <v>1411445.207473977</v>
+        <v>1138679.211787854</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -24689,7 +24689,7 @@
         <v>45932</v>
       </c>
       <c r="B99">
-        <v>1411730.644402237</v>
+        <v>1138702.994712988</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -24697,7 +24697,7 @@
         <v>45933</v>
       </c>
       <c r="B100">
-        <v>1418786.703604664</v>
+        <v>1142910.238027842</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -24705,7 +24705,7 @@
         <v>45936</v>
       </c>
       <c r="B101">
-        <v>1422776.101604664</v>
+        <v>1146183.953027842</v>
       </c>
     </row>
   </sheetData>

</xml_diff>